<commit_message>
Omitted pooled samples and updated Zn toxicity plots
</commit_message>
<xml_diff>
--- a/Zinc/4. Exploratory data analysis/Normality_checks.xlsx
+++ b/Zinc/4. Exploratory data analysis/Normality_checks.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -167,7 +167,10 @@
     <t xml:space="preserve">TOrg_K_M</t>
   </si>
   <si>
-    <t xml:space="preserve">Zn_Toxicity_Daphnia_M</t>
+    <t xml:space="preserve">Zn_chronic_tox_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zn_acute_tox_M</t>
   </si>
   <si>
     <t xml:space="preserve">DOC_M</t>
@@ -374,10 +377,16 @@
     <t xml:space="preserve">TOrg_K_nM</t>
   </si>
   <si>
-    <t xml:space="preserve">Zn_Toxicity_Daphnia_uM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zn_Toxicity_Daphnia_nM</t>
+    <t xml:space="preserve">Zn_chronic_tox_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zn_chronic_tox_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zn_acute_tox_uM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zn_acute_tox_nM</t>
   </si>
   <si>
     <t xml:space="preserve">BL_Zn_nmol_kg</t>
@@ -1297,7 +1306,7 @@
         <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>0.32054073838517</v>
+        <v>1.09014872856816</v>
       </c>
     </row>
     <row r="49">
@@ -1308,7 +1317,7 @@
         <v>4</v>
       </c>
       <c r="C49" t="n">
-        <v>3.92701712304009</v>
+        <v>0.527955794767177</v>
       </c>
     </row>
     <row r="50">
@@ -1330,7 +1339,7 @@
         <v>4</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.534352395703903</v>
+        <v>3.92701712304009</v>
       </c>
     </row>
     <row r="52">
@@ -1341,7 +1350,7 @@
         <v>4</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.534352395703905</v>
+        <v>-0.534352395703903</v>
       </c>
     </row>
     <row r="53">
@@ -1352,7 +1361,7 @@
         <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>-0.296160296305932</v>
+        <v>-0.534352395703905</v>
       </c>
     </row>
     <row r="54">
@@ -1363,7 +1372,7 @@
         <v>4</v>
       </c>
       <c r="C54" t="n">
-        <v>-0.296160296305931</v>
+        <v>-0.296160296305932</v>
       </c>
     </row>
     <row r="55">
@@ -1374,7 +1383,7 @@
         <v>4</v>
       </c>
       <c r="C55" t="n">
-        <v>1.66356916338087</v>
+        <v>-0.296160296305931</v>
       </c>
     </row>
     <row r="56">
@@ -1396,7 +1405,7 @@
         <v>4</v>
       </c>
       <c r="C57" t="n">
-        <v>2.01866181190736</v>
+        <v>1.66356916338087</v>
       </c>
     </row>
     <row r="58">
@@ -1418,7 +1427,7 @@
         <v>4</v>
       </c>
       <c r="C59" t="n">
-        <v>1.11838120514126</v>
+        <v>2.01866181190736</v>
       </c>
     </row>
     <row r="60">
@@ -1440,7 +1449,7 @@
         <v>4</v>
       </c>
       <c r="C61" t="n">
-        <v>2.1535439501211</v>
+        <v>1.11838120514126</v>
       </c>
     </row>
     <row r="62">
@@ -1462,7 +1471,7 @@
         <v>4</v>
       </c>
       <c r="C63" t="n">
-        <v>-0.614198152259787</v>
+        <v>2.1535439501211</v>
       </c>
     </row>
     <row r="64">
@@ -1484,7 +1493,7 @@
         <v>4</v>
       </c>
       <c r="C65" t="n">
-        <v>2.27374916500553</v>
+        <v>-0.614198152259787</v>
       </c>
     </row>
     <row r="66">
@@ -1506,7 +1515,7 @@
         <v>4</v>
       </c>
       <c r="C67" t="n">
-        <v>4.25239757909376</v>
+        <v>2.27374916500553</v>
       </c>
     </row>
     <row r="68">
@@ -1528,7 +1537,7 @@
         <v>4</v>
       </c>
       <c r="C69" t="n">
-        <v>2.49729594453213</v>
+        <v>4.25239757909376</v>
       </c>
     </row>
     <row r="70">
@@ -1550,7 +1559,7 @@
         <v>4</v>
       </c>
       <c r="C71" t="n">
-        <v>6.188471916066</v>
+        <v>2.49729594453213</v>
       </c>
     </row>
     <row r="72">
@@ -1572,7 +1581,7 @@
         <v>4</v>
       </c>
       <c r="C73" t="n">
-        <v>9.22841682466233</v>
+        <v>6.188471916066</v>
       </c>
     </row>
     <row r="74">
@@ -1594,7 +1603,7 @@
         <v>4</v>
       </c>
       <c r="C75" t="n">
-        <v>6.43827227328214</v>
+        <v>9.22841682466233</v>
       </c>
     </row>
     <row r="76">
@@ -1616,7 +1625,7 @@
         <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>2.1996824357861</v>
+        <v>6.43827227328214</v>
       </c>
     </row>
     <row r="78">
@@ -1638,7 +1647,7 @@
         <v>4</v>
       </c>
       <c r="C79" t="n">
-        <v>2.51233871275674</v>
+        <v>2.1996824357861</v>
       </c>
     </row>
     <row r="80">
@@ -1660,7 +1669,7 @@
         <v>4</v>
       </c>
       <c r="C81" t="n">
-        <v>4.4358300437397</v>
+        <v>2.51233871275674</v>
       </c>
     </row>
     <row r="82">
@@ -1682,7 +1691,7 @@
         <v>4</v>
       </c>
       <c r="C83" t="n">
-        <v>-10.1871446959223</v>
+        <v>4.4358300437397</v>
       </c>
     </row>
     <row r="84">
@@ -1693,7 +1702,7 @@
         <v>4</v>
       </c>
       <c r="C84" t="n">
-        <v>-10.1871446959219</v>
+        <v>-10.1871446959223</v>
       </c>
     </row>
     <row r="85">
@@ -1704,7 +1713,7 @@
         <v>4</v>
       </c>
       <c r="C85" t="n">
-        <v>2.23383168486604</v>
+        <v>-10.1871446959219</v>
       </c>
     </row>
     <row r="86">
@@ -1726,7 +1735,7 @@
         <v>4</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.664546207661824</v>
+        <v>2.23383168486604</v>
       </c>
     </row>
     <row r="88">
@@ -1737,7 +1746,7 @@
         <v>4</v>
       </c>
       <c r="C88" t="n">
-        <v>-0.664546207661826</v>
+        <v>-0.664546207661824</v>
       </c>
     </row>
     <row r="89">
@@ -1748,7 +1757,7 @@
         <v>4</v>
       </c>
       <c r="C89" t="n">
-        <v>2.47411042756224</v>
+        <v>-0.664546207661826</v>
       </c>
     </row>
     <row r="90">
@@ -1770,7 +1779,7 @@
         <v>4</v>
       </c>
       <c r="C91" t="n">
-        <v>16.4218761825449</v>
+        <v>2.47411042756224</v>
       </c>
     </row>
     <row r="92">
@@ -1792,7 +1801,7 @@
         <v>4</v>
       </c>
       <c r="C93" t="n">
-        <v>12.5888727271132</v>
+        <v>16.4218761825449</v>
       </c>
     </row>
     <row r="94">
@@ -1814,7 +1823,7 @@
         <v>4</v>
       </c>
       <c r="C95" t="n">
-        <v>0.252829596764858</v>
+        <v>12.5888727271132</v>
       </c>
     </row>
     <row r="96">
@@ -1825,7 +1834,7 @@
         <v>4</v>
       </c>
       <c r="C96" t="n">
-        <v>0.252829596764857</v>
+        <v>0.252829596764858</v>
       </c>
     </row>
     <row r="97">
@@ -1836,7 +1845,7 @@
         <v>4</v>
       </c>
       <c r="C97" t="n">
-        <v>7.37478377102132</v>
+        <v>0.252829596764857</v>
       </c>
     </row>
     <row r="98">
@@ -1858,7 +1867,7 @@
         <v>4</v>
       </c>
       <c r="C99" t="n">
-        <v>1.77298331310007</v>
+        <v>7.37478377102132</v>
       </c>
     </row>
     <row r="100">
@@ -1880,7 +1889,7 @@
         <v>4</v>
       </c>
       <c r="C101" t="n">
-        <v>0.174548980742532</v>
+        <v>1.77298331310007</v>
       </c>
     </row>
     <row r="102">
@@ -1902,7 +1911,7 @@
         <v>4</v>
       </c>
       <c r="C103" t="n">
-        <v>7.2070761259635</v>
+        <v>0.174548980742532</v>
       </c>
     </row>
     <row r="104">
@@ -1924,7 +1933,7 @@
         <v>4</v>
       </c>
       <c r="C105" t="n">
-        <v>1.004676147866</v>
+        <v>7.2070761259635</v>
       </c>
     </row>
     <row r="106">
@@ -1946,7 +1955,7 @@
         <v>4</v>
       </c>
       <c r="C107" t="n">
-        <v>4.28909721799728</v>
+        <v>1.004676147866</v>
       </c>
     </row>
     <row r="108">
@@ -1968,7 +1977,7 @@
         <v>4</v>
       </c>
       <c r="C109" t="n">
-        <v>3.2584891927878</v>
+        <v>4.28909721799728</v>
       </c>
     </row>
     <row r="110">
@@ -1990,7 +1999,7 @@
         <v>4</v>
       </c>
       <c r="C111" t="n">
-        <v>3.46625703766325</v>
+        <v>3.2584891927878</v>
       </c>
     </row>
     <row r="112">
@@ -2012,7 +2021,7 @@
         <v>4</v>
       </c>
       <c r="C113" t="n">
-        <v>13.6543329574097</v>
+        <v>3.46625703766325</v>
       </c>
     </row>
     <row r="114">
@@ -2034,7 +2043,7 @@
         <v>4</v>
       </c>
       <c r="C115" t="n">
-        <v>16.4207020886032</v>
+        <v>13.6543329574097</v>
       </c>
     </row>
     <row r="116">
@@ -2056,7 +2065,7 @@
         <v>4</v>
       </c>
       <c r="C117" t="n">
-        <v>0.320540738385171</v>
+        <v>16.4207020886032</v>
       </c>
     </row>
     <row r="118">
@@ -2067,7 +2076,7 @@
         <v>4</v>
       </c>
       <c r="C118" t="n">
-        <v>0.320540738385171</v>
+        <v>1.09014872856816</v>
       </c>
     </row>
     <row r="119">
@@ -2078,7 +2087,7 @@
         <v>4</v>
       </c>
       <c r="C119" t="n">
-        <v>5.18284830037465</v>
+        <v>1.09014872856815</v>
       </c>
     </row>
     <row r="120">
@@ -2089,7 +2098,7 @@
         <v>4</v>
       </c>
       <c r="C120" t="n">
-        <v>5.18284830037465</v>
+        <v>0.527955794767177</v>
       </c>
     </row>
     <row r="121">
@@ -2100,7 +2109,7 @@
         <v>4</v>
       </c>
       <c r="C121" t="n">
-        <v>5.18284830037465</v>
+        <v>0.527955794767177</v>
       </c>
     </row>
     <row r="122">
@@ -2111,7 +2120,7 @@
         <v>4</v>
       </c>
       <c r="C122" t="n">
-        <v>-2.82360964163951</v>
+        <v>5.18284830037465</v>
       </c>
     </row>
     <row r="123">
@@ -2122,7 +2131,7 @@
         <v>4</v>
       </c>
       <c r="C123" t="n">
-        <v>-2.82360964163951</v>
+        <v>5.18284830037465</v>
       </c>
     </row>
     <row r="124">
@@ -2133,7 +2142,7 @@
         <v>4</v>
       </c>
       <c r="C124" t="n">
-        <v>-2.82360964163951</v>
+        <v>5.18284830037465</v>
       </c>
     </row>
     <row r="125">
@@ -2144,7 +2153,7 @@
         <v>4</v>
       </c>
       <c r="C125" t="n">
-        <v>10.8005922632227</v>
+        <v>-2.82360964163951</v>
       </c>
     </row>
     <row r="126">
@@ -2155,7 +2164,7 @@
         <v>4</v>
       </c>
       <c r="C126" t="n">
-        <v>10.8005922632227</v>
+        <v>-2.82360964163951</v>
       </c>
     </row>
     <row r="127">
@@ -2166,7 +2175,7 @@
         <v>4</v>
       </c>
       <c r="C127" t="n">
-        <v>10.8005922632227</v>
+        <v>-2.82360964163951</v>
       </c>
     </row>
     <row r="128">
@@ -2174,10 +2183,10 @@
         <v>131</v>
       </c>
       <c r="B128" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C128" t="n">
-        <v>0.202544678355585</v>
+        <v>10.8005922632227</v>
       </c>
     </row>
     <row r="129">
@@ -2185,10 +2194,10 @@
         <v>132</v>
       </c>
       <c r="B129" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C129" t="n">
-        <v>0.202544678355585</v>
+        <v>10.8005922632227</v>
       </c>
     </row>
     <row r="130">
@@ -2196,10 +2205,10 @@
         <v>133</v>
       </c>
       <c r="B130" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C130" t="n">
-        <v>0.202544678355585</v>
+        <v>10.8005922632227</v>
       </c>
     </row>
     <row r="131">
@@ -2207,10 +2216,10 @@
         <v>134</v>
       </c>
       <c r="B131" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C131" t="n">
-        <v>1.84471536408702</v>
+        <v>0.202544678355585</v>
       </c>
     </row>
     <row r="132">
@@ -2218,10 +2227,10 @@
         <v>135</v>
       </c>
       <c r="B132" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C132" t="n">
-        <v>1.84471536408702</v>
+        <v>0.202544678355585</v>
       </c>
     </row>
     <row r="133">
@@ -2229,10 +2238,10 @@
         <v>136</v>
       </c>
       <c r="B133" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C133" t="n">
-        <v>1.84471536408701</v>
+        <v>0.202544678355585</v>
       </c>
     </row>
     <row r="134">
@@ -2243,7 +2252,7 @@
         <v>4</v>
       </c>
       <c r="C134" t="n">
-        <v>6.17281251617355</v>
+        <v>1.84471536408702</v>
       </c>
     </row>
     <row r="135">
@@ -2254,7 +2263,7 @@
         <v>4</v>
       </c>
       <c r="C135" t="n">
-        <v>6.17281251617355</v>
+        <v>1.84471536408702</v>
       </c>
     </row>
     <row r="136">
@@ -2265,7 +2274,7 @@
         <v>4</v>
       </c>
       <c r="C136" t="n">
-        <v>6.17281251617355</v>
+        <v>1.84471536408701</v>
       </c>
     </row>
     <row r="137">
@@ -2276,7 +2285,7 @@
         <v>4</v>
       </c>
       <c r="C137" t="n">
-        <v>4.06385953609146</v>
+        <v>6.17281251617355</v>
       </c>
     </row>
     <row r="138">
@@ -2287,7 +2296,7 @@
         <v>4</v>
       </c>
       <c r="C138" t="n">
-        <v>4.06385953609146</v>
+        <v>6.17281251617355</v>
       </c>
     </row>
     <row r="139">
@@ -2298,7 +2307,7 @@
         <v>4</v>
       </c>
       <c r="C139" t="n">
-        <v>4.06385953609146</v>
+        <v>6.17281251617355</v>
       </c>
     </row>
     <row r="140">
@@ -2309,6 +2318,39 @@
         <v>4</v>
       </c>
       <c r="C140" t="n">
+        <v>4.06385953609146</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>144</v>
+      </c>
+      <c r="B141" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" t="n">
+        <v>4.06385953609146</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>145</v>
+      </c>
+      <c r="B142" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" t="n">
+        <v>4.06385953609146</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>146</v>
+      </c>
+      <c r="B143" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" t="n">
         <v>0.9091030094148</v>
       </c>
     </row>

</xml_diff>